<commit_message>
feat: implement Requisition-side AKD/AKL/NIE data foundation
- Add AkdAklDeclaration enum to represent customer declaration status.
- Extend CalibrationRequestItem model to include akdAkl and akdAklDeclaration fields.
- Update Zod schemas for input validation and API contracts to include new fields.
- Modify API service methods to handle new fields during create and update operations.
- Ensure Excel import functionality supports optional AKD/AKL/NIE values without breaking existing behavior.
- Document changes in implementation reports and API contract references.
</commit_message>
<xml_diff>
--- a/apps/portal/public/medcal-requisition-template.xlsx
+++ b/apps/portal/public/medcal-requisition-template.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="27">
   <si>
     <t>Nama Alat</t>
   </si>
@@ -26,6 +26,9 @@
     <t>Device ID</t>
   </si>
   <si>
+    <t>AKD/AKL/NIE</t>
+  </si>
+  <si>
     <t>Contoh: Tensimeter</t>
   </si>
   <si>
@@ -47,6 +50,9 @@
     <t>Contoh: Dental Unit</t>
   </si>
   <si>
+    <t>AKD 20403012345</t>
+  </si>
+  <si>
     <t>Hapus baris contoh di atas, lalu isi data alat customer mulai dari sini.</t>
   </si>
   <si>
@@ -68,10 +74,16 @@
     <t>• Device ID  : OPSIONAL. Isi hanya jika customer memberikan Device ID. Satu baris hanya boleh berisi satu Device ID.</t>
   </si>
   <si>
+    <t>• AKD/AKL/NIE: OPSIONAL. Nomor Izin Edar yang diberikan customer (maks. 120 karakter). Boleh diisi untuk Qty berapa pun. Kosongkan jika customer belum memberikan.</t>
+  </si>
+  <si>
     <t>Aturan penting:</t>
   </si>
   <si>
     <t>• Setiap baris Excel menjadi 1 item requisition. Qty tetap tersimpan sebagai jumlah unit pada item tersebut — baris TIDAK dipecah menjadi beberapa item.</t>
+  </si>
+  <si>
+    <t>• AKD/AKL/NIE yang diisi adalah deklarasi customer, bukan hasil verifikasi teknis per unit fisik. Verifikasi final per unit dilakukan kemudian oleh Teknisi.</t>
   </si>
   <si>
     <t>• Jangan invent/membuat placeholder Device ID.</t>
@@ -472,16 +484,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="10" customWidth="1"/>
     <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -494,60 +507,73 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2">
         <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+      <c r="E2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C3">
         <v>3</v>
       </c>
       <c r="D3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+      <c r="E3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+      <c r="E4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A5:E5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -556,7 +582,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="100" customWidth="1"/>
@@ -564,72 +590,82 @@
   <sheetData>
     <row r="1" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>19</v>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>6</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>22</v>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>